<commit_message>
0.5.8 - NASA Medical Requirements
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-aerospace-behavioral-state-cs.xlsx
+++ b/docs/CodeSystem-aerospace-behavioral-state-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.5.6</t>
+    <t>0.5.8</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-30T19:11:20-07:00</t>
+    <t>2026-02-02T11:11:20-06:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Add citations, restructure navigation, and bump version to 0.6.0
Add AsMA 2026 CMS-formatted references to abstracts page, add FHIR
artifact hyperlinks across pagecontent files, create new hyperbaric
medicine page, rename neutral-buoyancy to scuba-training with expanded
content, restructure sushi-config menu for better organization, and
update terminology ndjson generation script.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-aerospace-behavioral-state-cs.xlsx
+++ b/docs/CodeSystem-aerospace-behavioral-state-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.5.12</t>
+    <t>0.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T00:24:16-05:00</t>
+    <t>2026-05-25T15:07:02-06:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>